<commit_message>
Complete Day 45 QA and remediation
</commit_message>
<xml_diff>
--- a/nifty100-financial-analysis(Bluestock-fintech)/Data/output/cashflow_intelligence.xlsx
+++ b/nifty100-financial-analysis(Bluestock-fintech)/Data/output/cashflow_intelligence.xlsx
@@ -517,7 +517,7 @@
         <v>0</v>
       </c>
       <c r="I2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -560,7 +560,7 @@
         <v>0</v>
       </c>
       <c r="I3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -607,7 +607,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="K4" t="n">
@@ -648,7 +648,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Excellent</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="K5" t="n">
@@ -687,7 +687,7 @@
         <v>0</v>
       </c>
       <c r="I6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -730,7 +730,7 @@
         <v>0</v>
       </c>
       <c r="I7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -845,11 +845,11 @@
         <v>0</v>
       </c>
       <c r="I10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="K10" t="n">
@@ -888,7 +888,7 @@
         <v>0</v>
       </c>
       <c r="I11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
@@ -931,11 +931,11 @@
         <v>0</v>
       </c>
       <c r="I12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="K12" t="n">
@@ -1017,7 +1017,7 @@
         <v>0</v>
       </c>
       <c r="I14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
@@ -1142,7 +1142,7 @@
         <v>0</v>
       </c>
       <c r="I17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
@@ -1228,7 +1228,7 @@
         <v>0</v>
       </c>
       <c r="I19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
@@ -1314,7 +1314,7 @@
         <v>0</v>
       </c>
       <c r="I21" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
@@ -1357,7 +1357,7 @@
         <v>0</v>
       </c>
       <c r="I22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
@@ -1400,7 +1400,7 @@
         <v>0</v>
       </c>
       <c r="I23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
@@ -1443,7 +1443,7 @@
         <v>0</v>
       </c>
       <c r="I24" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
@@ -1570,7 +1570,7 @@
         <v>0</v>
       </c>
       <c r="I27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
@@ -1613,7 +1613,7 @@
         <v>0</v>
       </c>
       <c r="I28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
@@ -1699,7 +1699,7 @@
         <v>0</v>
       </c>
       <c r="I30" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
@@ -1742,7 +1742,7 @@
         <v>0</v>
       </c>
       <c r="I31" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
@@ -1785,7 +1785,7 @@
         <v>0</v>
       </c>
       <c r="I32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
@@ -1828,7 +1828,7 @@
         <v>0</v>
       </c>
       <c r="I33" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J33" t="inlineStr">
         <is>
@@ -1871,7 +1871,7 @@
         <v>0</v>
       </c>
       <c r="I34" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J34" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
         <v>0</v>
       </c>
       <c r="I37" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J37" t="inlineStr">
         <is>
@@ -2127,11 +2127,11 @@
         <v>0</v>
       </c>
       <c r="I40" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Excellent</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="K40" t="n">
@@ -2170,7 +2170,7 @@
         <v>0</v>
       </c>
       <c r="I41" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J41" t="inlineStr">
         <is>
@@ -2213,11 +2213,11 @@
         <v>0</v>
       </c>
       <c r="I42" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="K42" t="n">
@@ -2256,7 +2256,7 @@
         <v>0</v>
       </c>
       <c r="I43" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J43" t="inlineStr">
         <is>
@@ -2299,7 +2299,7 @@
         <v>0</v>
       </c>
       <c r="I44" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J44" t="inlineStr">
         <is>
@@ -2385,11 +2385,11 @@
         <v>0</v>
       </c>
       <c r="I46" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>Excellent</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="K46" t="n">
@@ -2428,7 +2428,7 @@
         <v>0</v>
       </c>
       <c r="I47" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J47" t="inlineStr">
         <is>
@@ -2471,7 +2471,7 @@
         <v>0</v>
       </c>
       <c r="I48" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J48" t="inlineStr">
         <is>
@@ -2514,7 +2514,7 @@
         <v>0</v>
       </c>
       <c r="I49" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J49" t="inlineStr">
         <is>
@@ -2557,7 +2557,7 @@
         <v>0</v>
       </c>
       <c r="I50" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J50" t="inlineStr">
         <is>
@@ -2598,7 +2598,7 @@
         <v>0</v>
       </c>
       <c r="I51" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J51" t="inlineStr">
         <is>
@@ -2727,7 +2727,7 @@
         <v>0</v>
       </c>
       <c r="I54" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J54" t="inlineStr">
         <is>
@@ -2770,7 +2770,7 @@
         <v>0</v>
       </c>
       <c r="I55" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J55" t="inlineStr">
         <is>
@@ -2856,7 +2856,7 @@
         <v>0</v>
       </c>
       <c r="I57" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J57" t="inlineStr">
         <is>
@@ -3028,7 +3028,7 @@
         <v>0</v>
       </c>
       <c r="I61" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J61" t="inlineStr">
         <is>
@@ -3071,7 +3071,7 @@
         <v>0</v>
       </c>
       <c r="I62" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J62" t="inlineStr">
         <is>
@@ -3114,7 +3114,7 @@
         <v>0</v>
       </c>
       <c r="I63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J63" t="inlineStr">
         <is>
@@ -3161,7 +3161,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="K64" t="n">
@@ -3241,11 +3241,11 @@
         <v>0</v>
       </c>
       <c r="I66" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>Excellent</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="K66" t="n">
@@ -3284,7 +3284,7 @@
         <v>0</v>
       </c>
       <c r="I67" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J67" t="inlineStr">
         <is>
@@ -3327,7 +3327,7 @@
         <v>0</v>
       </c>
       <c r="I68" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J68" t="inlineStr">
         <is>
@@ -3370,7 +3370,7 @@
         <v>0</v>
       </c>
       <c r="I69" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J69" t="inlineStr">
         <is>
@@ -3413,7 +3413,7 @@
         <v>0</v>
       </c>
       <c r="I70" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J70" t="inlineStr">
         <is>
@@ -3456,7 +3456,7 @@
         <v>0</v>
       </c>
       <c r="I71" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J71" t="inlineStr">
         <is>
@@ -3540,7 +3540,7 @@
         <v>0</v>
       </c>
       <c r="I73" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J73" t="inlineStr">
         <is>
@@ -3667,7 +3667,7 @@
         <v>0</v>
       </c>
       <c r="I76" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J76" t="inlineStr">
         <is>
@@ -3796,11 +3796,11 @@
         <v>0</v>
       </c>
       <c r="I79" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="K79" t="n">
@@ -3962,7 +3962,7 @@
         <v>0</v>
       </c>
       <c r="I83" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J83" t="inlineStr">
         <is>
@@ -4017,11 +4017,11 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>1.0364</v>
+        <v>0.9893</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>High Quality</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -4033,16 +4033,16 @@
         </is>
       </c>
       <c r="F85" t="n">
-        <v>9.82</v>
+        <v>13.41</v>
       </c>
       <c r="G85" t="n">
-        <v>83.08</v>
+        <v>109.39</v>
       </c>
       <c r="H85" t="b">
         <v>0</v>
       </c>
       <c r="I85" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J85" t="inlineStr">
         <is>
@@ -4089,7 +4089,7 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="K86" t="n">
@@ -4128,7 +4128,7 @@
         <v>0</v>
       </c>
       <c r="I87" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J87" t="inlineStr">
         <is>
@@ -4171,7 +4171,7 @@
         <v>0</v>
       </c>
       <c r="I88" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J88" t="inlineStr">
         <is>
@@ -4212,7 +4212,7 @@
         <v>0</v>
       </c>
       <c r="I89" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J89" t="inlineStr">
         <is>
@@ -4255,11 +4255,11 @@
         <v>0</v>
       </c>
       <c r="I90" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="K90" t="n">
@@ -4298,7 +4298,7 @@
         <v>0</v>
       </c>
       <c r="I91" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J91" t="inlineStr">
         <is>
@@ -4341,7 +4341,7 @@
         <v>0</v>
       </c>
       <c r="I92" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J92" t="inlineStr">
         <is>
@@ -4384,7 +4384,7 @@
         <v>0</v>
       </c>
       <c r="I93" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J93" t="inlineStr">
         <is>

</xml_diff>